<commit_message>
Mejora visual del dasboard
</commit_message>
<xml_diff>
--- a/data/gastos.xlsx
+++ b/data/gastos.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1399,9 +1399,269 @@
         <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51">
+        <v>1772346830342</v>
+      </c>
+      <c r="B51" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Julian</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E51">
+        <v>80000</v>
+      </c>
+      <c r="F51" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>1772346841923</v>
+      </c>
+      <c r="B52" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Martha Arias</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E52">
+        <v>80000</v>
+      </c>
+      <c r="F52" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>1772346877948</v>
+      </c>
+      <c r="B53" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Juanita Salazar</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E53">
+        <v>70000</v>
+      </c>
+      <c r="F53" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>1772346890728</v>
+      </c>
+      <c r="B54" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Valeria Valencia</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E54">
+        <v>70000</v>
+      </c>
+      <c r="F54" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>1772346899643</v>
+      </c>
+      <c r="B55" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Laura Cardona</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E55">
+        <v>70000</v>
+      </c>
+      <c r="F55" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>1772346909031</v>
+      </c>
+      <c r="B56" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Jhojan Buitrago</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E56">
+        <v>70000</v>
+      </c>
+      <c r="F56" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>1772346968903</v>
+      </c>
+      <c r="B57" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Alexander Castaño</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E57">
+        <v>70000</v>
+      </c>
+      <c r="F57" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>1772346978406</v>
+      </c>
+      <c r="B58" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Fredy Arias</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E58">
+        <v>70000</v>
+      </c>
+      <c r="F58" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>1772346986834</v>
+      </c>
+      <c r="B59" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Dreisy Gamarra</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E59">
+        <v>80000</v>
+      </c>
+      <c r="F59" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>1772346998145</v>
+      </c>
+      <c r="B60" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C60" t="str">
+        <v xml:space="preserve">Juan Carlos </v>
+      </c>
+      <c r="D60" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E60">
+        <v>80000</v>
+      </c>
+      <c r="F60" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>1772347008167</v>
+      </c>
+      <c r="B61" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C61" t="str">
+        <v xml:space="preserve">Sebastian Alzate </v>
+      </c>
+      <c r="D61" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E61">
+        <v>150000</v>
+      </c>
+      <c r="F61" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>1772347035207</v>
+      </c>
+      <c r="B62" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Luisa Vallejo</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E62">
+        <v>80000</v>
+      </c>
+      <c r="F62" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>1772347102598</v>
+      </c>
+      <c r="B63" t="str">
+        <v>2026-02-28</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Limones- Bolsas para basura</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Insumos</v>
+      </c>
+      <c r="E63">
+        <v>20000</v>
+      </c>
+      <c r="F63" t="str">
+        <v>{"nombre":"Luisa","rol":"ADMIN"}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F63"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se incluye en el modulo de gastos la opcion de descarga y se generaopcion de filtros
</commit_message>
<xml_diff>
--- a/data/gastos.xlsx
+++ b/data/gastos.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F127"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2299,9 +2299,649 @@
         <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
       </c>
     </row>
+    <row r="96">
+      <c r="A96">
+        <v>1774649419520</v>
+      </c>
+      <c r="B96" t="str">
+        <v>2026-03-27</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Pago Luz</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Servicios</v>
+      </c>
+      <c r="E96">
+        <v>550355</v>
+      </c>
+      <c r="F96" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97">
+        <v>1774666888081</v>
+      </c>
+      <c r="B97" t="str">
+        <v>2026-03-27</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Luz Helena</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E97">
+        <v>100000</v>
+      </c>
+      <c r="F97" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98">
+        <v>1774666898706</v>
+      </c>
+      <c r="B98" t="str">
+        <v>2026-03-27</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Fredy</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E98">
+        <v>80000</v>
+      </c>
+      <c r="F98" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99">
+        <v>1774666909157</v>
+      </c>
+      <c r="B99" t="str">
+        <v>2026-03-27</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Luisa</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E99">
+        <v>80000</v>
+      </c>
+      <c r="F99" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100">
+        <v>1774668119905</v>
+      </c>
+      <c r="B100" t="str">
+        <v>2026-03-27</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Bailarin</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E100">
+        <v>20000</v>
+      </c>
+      <c r="F100" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101">
+        <v>1774668145713</v>
+      </c>
+      <c r="B101" t="str">
+        <v>2026-03-27</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Zumo de limon, Hielo</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Insumos</v>
+      </c>
+      <c r="E101">
+        <v>96000</v>
+      </c>
+      <c r="F101" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102">
+        <v>1774766331088</v>
+      </c>
+      <c r="B102" t="str">
+        <v>2026-03-28</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Julian</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E102">
+        <v>80000</v>
+      </c>
+      <c r="F102" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103">
+        <v>1774766338551</v>
+      </c>
+      <c r="B103" t="str">
+        <v>2026-03-28</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Martha</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E103">
+        <v>80000</v>
+      </c>
+      <c r="F103" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104">
+        <v>1774766345858</v>
+      </c>
+      <c r="B104" t="str">
+        <v>2026-03-28</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Valeria</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E104">
+        <v>70000</v>
+      </c>
+      <c r="F104" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105">
+        <v>1774766352070</v>
+      </c>
+      <c r="B105" t="str">
+        <v>2026-03-28</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Juanita</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E105">
+        <v>70000</v>
+      </c>
+      <c r="F105" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106">
+        <v>1774766358724</v>
+      </c>
+      <c r="B106" t="str">
+        <v>2026-03-28</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Saray</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E106">
+        <v>70000</v>
+      </c>
+      <c r="F106" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107">
+        <v>1774766368874</v>
+      </c>
+      <c r="B107" t="str">
+        <v>2026-03-28</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Dreisy</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E107">
+        <v>80000</v>
+      </c>
+      <c r="F107" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108">
+        <v>1774766378468</v>
+      </c>
+      <c r="B108" t="str">
+        <v>2026-03-28</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Luisa</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E108">
+        <v>80000</v>
+      </c>
+      <c r="F108" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109">
+        <v>1774766387936</v>
+      </c>
+      <c r="B109" t="str">
+        <v>2026-03-28</v>
+      </c>
+      <c r="C109" t="str">
+        <v>Alexander</v>
+      </c>
+      <c r="D109" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E109">
+        <v>70000</v>
+      </c>
+      <c r="F109" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110">
+        <v>1774766398851</v>
+      </c>
+      <c r="B110" t="str">
+        <v>2026-03-28</v>
+      </c>
+      <c r="C110" t="str">
+        <v>Fredy</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E110">
+        <v>70000</v>
+      </c>
+      <c r="F110" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111">
+        <v>1774766407234</v>
+      </c>
+      <c r="B111" t="str">
+        <v>2026-03-28</v>
+      </c>
+      <c r="C111" t="str">
+        <v>Juan Carlos</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E111">
+        <v>80000</v>
+      </c>
+      <c r="F111" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112">
+        <v>1774766418227</v>
+      </c>
+      <c r="B112" t="str">
+        <v>2026-03-28</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Sebastian</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E112">
+        <v>150000</v>
+      </c>
+      <c r="F112" t="str">
+        <v>{"nombre":"Luisa-Dreisy","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113">
+        <v>1775095158198</v>
+      </c>
+      <c r="B113" t="str">
+        <v>2026-04-02</v>
+      </c>
+      <c r="C113" t="str">
+        <v>taxy dancer kiko</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E113">
+        <v>20000</v>
+      </c>
+      <c r="F113" t="str">
+        <v>{"nombre":"juan","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114">
+        <v>1775097073345</v>
+      </c>
+      <c r="B114" t="str">
+        <v>2026-04-02</v>
+      </c>
+      <c r="C114" t="str">
+        <v>Sebastian</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E114">
+        <v>80000</v>
+      </c>
+      <c r="F114" t="str">
+        <v>{"nombre":"juan","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115">
+        <v>1775097096162</v>
+      </c>
+      <c r="B115" t="str">
+        <v>2026-04-02</v>
+      </c>
+      <c r="C115" t="str">
+        <v>Stiven</v>
+      </c>
+      <c r="D115" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E115">
+        <v>70000</v>
+      </c>
+      <c r="F115" t="str">
+        <v>{"nombre":"juan","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116">
+        <v>1775097588042</v>
+      </c>
+      <c r="B116" t="str">
+        <v>2026-04-01</v>
+      </c>
+      <c r="C116" t="str">
+        <v>Juan</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E116">
+        <v>80000</v>
+      </c>
+      <c r="F116" t="str">
+        <v>{"nombre":"juan","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117">
+        <v>1775356873388</v>
+      </c>
+      <c r="B117" t="str">
+        <v>2026-04-04</v>
+      </c>
+      <c r="C117" t="str">
+        <v>Compra hielo</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E117">
+        <v>66000</v>
+      </c>
+      <c r="F117" t="str">
+        <v>{"nombre":"Dianis","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118">
+        <v>1775371919048</v>
+      </c>
+      <c r="B118" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="C118" t="str">
+        <v>Alexander (Mesero)</v>
+      </c>
+      <c r="D118" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E118">
+        <v>70000</v>
+      </c>
+      <c r="F118" t="str">
+        <v>{"nombre":"Dianis","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119">
+        <v>1775371939195</v>
+      </c>
+      <c r="B119" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="C119" t="str">
+        <v>Saray  (Mesero)</v>
+      </c>
+      <c r="D119" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E119">
+        <v>70000</v>
+      </c>
+      <c r="F119" t="str">
+        <v>{"nombre":"Dianis","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120">
+        <v>1775371955898</v>
+      </c>
+      <c r="B120" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="C120" t="str">
+        <v>Juanita  (Mesero)</v>
+      </c>
+      <c r="D120" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E120">
+        <v>70000</v>
+      </c>
+      <c r="F120" t="str">
+        <v>{"nombre":"Dianis","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121">
+        <v>1775371970555</v>
+      </c>
+      <c r="B121" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="C121" t="str">
+        <v>Johan  (Mesero)</v>
+      </c>
+      <c r="D121" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E121">
+        <v>70000</v>
+      </c>
+      <c r="F121" t="str">
+        <v>{"nombre":"Dianis","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122">
+        <v>1775371993421</v>
+      </c>
+      <c r="B122" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="C122" t="str">
+        <v>Martha C  (Mesero)</v>
+      </c>
+      <c r="D122" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E122">
+        <v>70000</v>
+      </c>
+      <c r="F122" t="str">
+        <v>{"nombre":"Dianis","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123">
+        <v>1775372016938</v>
+      </c>
+      <c r="B123" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Juan Carlos (Barra)</v>
+      </c>
+      <c r="D123" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E123">
+        <v>80000</v>
+      </c>
+      <c r="F123" t="str">
+        <v>{"nombre":"Dianis","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124">
+        <v>1775372037261</v>
+      </c>
+      <c r="B124" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="C124" t="str">
+        <v>Stiven (Barra)</v>
+      </c>
+      <c r="D124" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E124">
+        <v>80000</v>
+      </c>
+      <c r="F124" t="str">
+        <v>{"nombre":"Dianis","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125">
+        <v>1775372053957</v>
+      </c>
+      <c r="B125" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="C125" t="str">
+        <v>Martha Arias (Puerta)</v>
+      </c>
+      <c r="D125" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E125">
+        <v>80000</v>
+      </c>
+      <c r="F125" t="str">
+        <v>{"nombre":"Dianis","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126">
+        <v>1775372076176</v>
+      </c>
+      <c r="B126" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="C126" t="str">
+        <v>Julian (Puerta)</v>
+      </c>
+      <c r="D126" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E126">
+        <v>80000</v>
+      </c>
+      <c r="F126" t="str">
+        <v>{"nombre":"Dianis","rol":"ADMIN"}</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127">
+        <v>1775372097746</v>
+      </c>
+      <c r="B127" t="str">
+        <v>2026-04-05</v>
+      </c>
+      <c r="C127" t="str">
+        <v>Sebastian (D.J)</v>
+      </c>
+      <c r="D127" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E127">
+        <v>150000</v>
+      </c>
+      <c r="F127" t="str">
+        <v>{"nombre":"Dianis","rol":"ADMIN"}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F95"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F127"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Extualizacion general del proyecto, cambio a tailwind css, revisin de responsividad, creacio de vista para catalogo y posteriormente ser implementado en QR
</commit_message>
<xml_diff>
--- a/data/gastos.xlsx
+++ b/data/gastos.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:F185"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2939,9 +2939,1169 @@
         <v>{"nombre":"Dianis","rol":"ADMIN"}</v>
       </c>
     </row>
+    <row r="128">
+      <c r="A128">
+        <v>1775682580741</v>
+      </c>
+      <c r="B128" t="str">
+        <v>2026-03-30</v>
+      </c>
+      <c r="C128" t="str">
+        <v>arriendo</v>
+      </c>
+      <c r="D128" t="str">
+        <v>Arriendo</v>
+      </c>
+      <c r="E128">
+        <v>6700000</v>
+      </c>
+      <c r="F128" t="str">
+        <v>Jorge</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129">
+        <v>1775686686783</v>
+      </c>
+      <c r="B129" t="str">
+        <v>2026-01-08</v>
+      </c>
+      <c r="C129" t="str">
+        <v>pago agua</v>
+      </c>
+      <c r="D129" t="str">
+        <v>Insumos</v>
+      </c>
+      <c r="E129">
+        <v>386134</v>
+      </c>
+      <c r="F129" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130">
+        <v>1775686780868</v>
+      </c>
+      <c r="B130" t="str">
+        <v>2026-01-08</v>
+      </c>
+      <c r="C130" t="str">
+        <v>pago luz</v>
+      </c>
+      <c r="D130" t="str">
+        <v>Servicios</v>
+      </c>
+      <c r="E130">
+        <v>662357</v>
+      </c>
+      <c r="F130" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131">
+        <v>1775687253560</v>
+      </c>
+      <c r="B131" t="str">
+        <v>2026-01-08</v>
+      </c>
+      <c r="C131" t="str">
+        <v>agua</v>
+      </c>
+      <c r="D131" t="str">
+        <v>Servicios</v>
+      </c>
+      <c r="E131">
+        <v>386134</v>
+      </c>
+      <c r="F131" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132">
+        <v>1775687585302</v>
+      </c>
+      <c r="B132" t="str">
+        <v>2026-01-08</v>
+      </c>
+      <c r="C132" t="str">
+        <v>arriendo</v>
+      </c>
+      <c r="D132" t="str">
+        <v>Arriendo</v>
+      </c>
+      <c r="E132">
+        <v>6296828</v>
+      </c>
+      <c r="F132" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133">
+        <v>1775687675799</v>
+      </c>
+      <c r="B133" t="str">
+        <v>2026-02-08</v>
+      </c>
+      <c r="C133" t="str">
+        <v>arriendo</v>
+      </c>
+      <c r="D133" t="str">
+        <v>Arriendo</v>
+      </c>
+      <c r="E133">
+        <v>6296828</v>
+      </c>
+      <c r="F133" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134">
+        <v>1775687767374</v>
+      </c>
+      <c r="B134" t="str">
+        <v>2026-01-08</v>
+      </c>
+      <c r="C134" t="str">
+        <v>internet</v>
+      </c>
+      <c r="D134" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E134">
+        <v>100000</v>
+      </c>
+      <c r="F134" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135">
+        <v>1775687893155</v>
+      </c>
+      <c r="B135" t="str">
+        <v>2026-02-08</v>
+      </c>
+      <c r="C135" t="str">
+        <v>internet</v>
+      </c>
+      <c r="D135" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E135">
+        <v>100000</v>
+      </c>
+      <c r="F135" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136">
+        <v>1775687893166</v>
+      </c>
+      <c r="B136" t="str">
+        <v>2026-02-08</v>
+      </c>
+      <c r="C136" t="str">
+        <v>internet</v>
+      </c>
+      <c r="D136" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E136">
+        <v>100000</v>
+      </c>
+      <c r="F136" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137">
+        <v>1775687958234</v>
+      </c>
+      <c r="B137" t="str">
+        <v>2026-03-08</v>
+      </c>
+      <c r="C137" t="str">
+        <v>internet</v>
+      </c>
+      <c r="D137" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E137">
+        <v>100000</v>
+      </c>
+      <c r="F137" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138">
+        <v>1775690022918</v>
+      </c>
+      <c r="B138" t="str">
+        <v>2026-02-08</v>
+      </c>
+      <c r="C138" t="str">
+        <v>caucho greca</v>
+      </c>
+      <c r="D138" t="str">
+        <v>Mantenimiento</v>
+      </c>
+      <c r="E138">
+        <v>5500</v>
+      </c>
+      <c r="F138" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139">
+        <v>1775690049371</v>
+      </c>
+      <c r="B139" t="str">
+        <v>2026-02-08</v>
+      </c>
+      <c r="C139" t="str">
+        <v>vasos</v>
+      </c>
+      <c r="D139" t="str">
+        <v>Insumos</v>
+      </c>
+      <c r="E139">
+        <v>150000</v>
+      </c>
+      <c r="F139" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140">
+        <v>1775690129239</v>
+      </c>
+      <c r="B140" t="str">
+        <v>2026-02-09</v>
+      </c>
+      <c r="C140" t="str">
+        <v>publicidad trompetas</v>
+      </c>
+      <c r="D140" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E140">
+        <v>500000</v>
+      </c>
+      <c r="F140" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141">
+        <v>1775690232276</v>
+      </c>
+      <c r="B141" t="str">
+        <v>2026-02-16</v>
+      </c>
+      <c r="C141" t="str">
+        <v>camara y comercio</v>
+      </c>
+      <c r="D141" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E141">
+        <v>200000</v>
+      </c>
+      <c r="F141" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142">
+        <v>1775690562600</v>
+      </c>
+      <c r="B142" t="str">
+        <v>2026-02-19</v>
+      </c>
+      <c r="C142" t="str">
+        <v>arreglo lampara mr tango</v>
+      </c>
+      <c r="D142" t="str">
+        <v>Mantenimiento</v>
+      </c>
+      <c r="E142">
+        <v>75000</v>
+      </c>
+      <c r="F142" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143">
+        <v>1775691305117</v>
+      </c>
+      <c r="B143" t="str">
+        <v>2026-01-19</v>
+      </c>
+      <c r="C143" t="str">
+        <v>aseo</v>
+      </c>
+      <c r="D143" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E143">
+        <v>400000</v>
+      </c>
+      <c r="F143" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144">
+        <v>1775691337012</v>
+      </c>
+      <c r="B144" t="str">
+        <v>2026-02-19</v>
+      </c>
+      <c r="C144" t="str">
+        <v>aseo trompeta</v>
+      </c>
+      <c r="D144" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E144">
+        <v>400000</v>
+      </c>
+      <c r="F144" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145">
+        <v>1775691360702</v>
+      </c>
+      <c r="B145" t="str">
+        <v>2026-03-19</v>
+      </c>
+      <c r="C145" t="str">
+        <v>aseo trompetas</v>
+      </c>
+      <c r="D145" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E145">
+        <v>400000</v>
+      </c>
+      <c r="F145" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146">
+        <v>1775691386866</v>
+      </c>
+      <c r="B146" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C146" t="str">
+        <v>aseo trompetas</v>
+      </c>
+      <c r="D146" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E146">
+        <v>400000</v>
+      </c>
+      <c r="F146" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147">
+        <v>1775691453355</v>
+      </c>
+      <c r="B147" t="str">
+        <v>2026-02-20</v>
+      </c>
+      <c r="C147" t="str">
+        <v>cables</v>
+      </c>
+      <c r="D147" t="str">
+        <v>Mantenimiento</v>
+      </c>
+      <c r="E147">
+        <v>15400</v>
+      </c>
+      <c r="F147" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148">
+        <v>1775691626175</v>
+      </c>
+      <c r="B148" t="str">
+        <v>2026-04-01</v>
+      </c>
+      <c r="C148" t="str">
+        <v>telrducha</v>
+      </c>
+      <c r="D148" t="str">
+        <v>Mantenimiento</v>
+      </c>
+      <c r="E148">
+        <v>9500</v>
+      </c>
+      <c r="F148" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149">
+        <v>1775870128796</v>
+      </c>
+      <c r="B149" t="str">
+        <v>2026-03-31</v>
+      </c>
+      <c r="C149" t="str">
+        <v>Gastos cafeteria</v>
+      </c>
+      <c r="D149" t="str">
+        <v>Cafeteria</v>
+      </c>
+      <c r="E149">
+        <v>150000</v>
+      </c>
+      <c r="F149" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150">
+        <v>1775870461228</v>
+      </c>
+      <c r="B150" t="str">
+        <v>2026-03-31</v>
+      </c>
+      <c r="C150" t="str">
+        <v>Barra en semana</v>
+      </c>
+      <c r="D150" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E150">
+        <v>1045000</v>
+      </c>
+      <c r="F150" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151">
+        <v>1775874794317</v>
+      </c>
+      <c r="B151" t="str">
+        <v>2026-03-31</v>
+      </c>
+      <c r="C151" t="str">
+        <v>Venta cafeteria</v>
+      </c>
+      <c r="D151" t="str">
+        <v>Cafeteria</v>
+      </c>
+      <c r="E151">
+        <v>4654000</v>
+      </c>
+      <c r="F151" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152">
+        <v>1775874908357</v>
+      </c>
+      <c r="B152" t="str">
+        <v>2026-04-10</v>
+      </c>
+      <c r="C152" t="str">
+        <v>Luz helena</v>
+      </c>
+      <c r="D152" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E152">
+        <v>100000</v>
+      </c>
+      <c r="F152" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153">
+        <v>1775874920128</v>
+      </c>
+      <c r="B153" t="str">
+        <v>2026-04-10</v>
+      </c>
+      <c r="C153" t="str">
+        <v>Fredy</v>
+      </c>
+      <c r="D153" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E153">
+        <v>80000</v>
+      </c>
+      <c r="F153" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154">
+        <v>1775874937839</v>
+      </c>
+      <c r="B154" t="str">
+        <v>2026-04-10</v>
+      </c>
+      <c r="C154" t="str">
+        <v>Luisa Vallejo</v>
+      </c>
+      <c r="D154" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E154">
+        <v>80000</v>
+      </c>
+      <c r="F154" t="str">
+        <v>Dianis</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155">
+        <v>1775960924723</v>
+      </c>
+      <c r="B155" t="str">
+        <v>2026-04-12</v>
+      </c>
+      <c r="C155" t="str">
+        <v>Hielo</v>
+      </c>
+      <c r="D155" t="str">
+        <v>Insumos</v>
+      </c>
+      <c r="E155">
+        <v>62000</v>
+      </c>
+      <c r="F155" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156">
+        <v>1776464098259</v>
+      </c>
+      <c r="B156" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="C156" t="str">
+        <v>Julian</v>
+      </c>
+      <c r="D156" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E156">
+        <v>80000</v>
+      </c>
+      <c r="F156" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157">
+        <v>1776464110007</v>
+      </c>
+      <c r="B157" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="C157" t="str">
+        <v>Martha</v>
+      </c>
+      <c r="D157" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E157">
+        <v>80000</v>
+      </c>
+      <c r="F157" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158">
+        <v>1776464125489</v>
+      </c>
+      <c r="B158" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="C158" t="str">
+        <v>Valeria</v>
+      </c>
+      <c r="D158" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E158">
+        <v>70000</v>
+      </c>
+      <c r="F158" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159">
+        <v>1776464134737</v>
+      </c>
+      <c r="B159" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="C159" t="str">
+        <v>Juanita</v>
+      </c>
+      <c r="D159" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E159">
+        <v>70000</v>
+      </c>
+      <c r="F159" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160">
+        <v>1776464144093</v>
+      </c>
+      <c r="B160" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="C160" t="str">
+        <v>Alexander</v>
+      </c>
+      <c r="D160" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E160">
+        <v>70000</v>
+      </c>
+      <c r="F160" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161">
+        <v>1776464153476</v>
+      </c>
+      <c r="B161" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="C161" t="str">
+        <v>Jhojan</v>
+      </c>
+      <c r="D161" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E161">
+        <v>70000</v>
+      </c>
+      <c r="F161" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162">
+        <v>1776464164556</v>
+      </c>
+      <c r="B162" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="C162" t="str">
+        <v>Martha 2</v>
+      </c>
+      <c r="D162" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E162">
+        <v>70000</v>
+      </c>
+      <c r="F162" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163">
+        <v>1776464308524</v>
+      </c>
+      <c r="B163" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="C163" t="str">
+        <v>Juan carlos</v>
+      </c>
+      <c r="D163" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E163">
+        <v>80000</v>
+      </c>
+      <c r="F163" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164">
+        <v>1776464332061</v>
+      </c>
+      <c r="B164" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="C164" t="str">
+        <v>Dreisy</v>
+      </c>
+      <c r="D164" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E164">
+        <v>80000</v>
+      </c>
+      <c r="F164" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165">
+        <v>1776464353809</v>
+      </c>
+      <c r="B165" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="C165" t="str">
+        <v>Sebastian</v>
+      </c>
+      <c r="D165" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E165">
+        <v>150000</v>
+      </c>
+      <c r="F165" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166">
+        <v>1776464364273</v>
+      </c>
+      <c r="B166" t="str">
+        <v>2026-04-11</v>
+      </c>
+      <c r="C166" t="str">
+        <v>Luisa</v>
+      </c>
+      <c r="D166" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E166">
+        <v>90000</v>
+      </c>
+      <c r="F166" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167">
+        <v>1776464378713</v>
+      </c>
+      <c r="B167" t="str">
+        <v>2026-04-17</v>
+      </c>
+      <c r="C167" t="str">
+        <v>Fredy</v>
+      </c>
+      <c r="D167" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E167">
+        <v>80000</v>
+      </c>
+      <c r="F167" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168">
+        <v>1776464392567</v>
+      </c>
+      <c r="B168" t="str">
+        <v>2026-04-17</v>
+      </c>
+      <c r="C168" t="str">
+        <v>Sebastian</v>
+      </c>
+      <c r="D168" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E168">
+        <v>100000</v>
+      </c>
+      <c r="F168" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169">
+        <v>1776464402060</v>
+      </c>
+      <c r="B169" t="str">
+        <v>2026-04-17</v>
+      </c>
+      <c r="C169" t="str">
+        <v>Luisa</v>
+      </c>
+      <c r="D169" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E169">
+        <v>80000</v>
+      </c>
+      <c r="F169" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170">
+        <v>1776473003853</v>
+      </c>
+      <c r="B170" t="str">
+        <v>2026-04-17</v>
+      </c>
+      <c r="C170" t="str">
+        <v>Agua</v>
+      </c>
+      <c r="D170" t="str">
+        <v>Servicios</v>
+      </c>
+      <c r="E170">
+        <v>427699</v>
+      </c>
+      <c r="F170" t="str">
+        <v>juan</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171">
+        <v>1776473429984</v>
+      </c>
+      <c r="B171" t="str">
+        <v>2026-04-17</v>
+      </c>
+      <c r="C171" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="D171" t="str">
+        <v>Insumos</v>
+      </c>
+      <c r="E171">
+        <v>158000</v>
+      </c>
+      <c r="F171" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172">
+        <v>1776480293747</v>
+      </c>
+      <c r="B172" t="str">
+        <v>2026-04-18</v>
+      </c>
+      <c r="C172" t="str">
+        <v>Cafeteria</v>
+      </c>
+      <c r="D172" t="str">
+        <v>Cafeteria</v>
+      </c>
+      <c r="E172">
+        <v>899000</v>
+      </c>
+      <c r="F172" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173">
+        <v>1776480422850</v>
+      </c>
+      <c r="B173" t="str">
+        <v>2026-04-18</v>
+      </c>
+      <c r="C173" t="str">
+        <v>Barra en semana</v>
+      </c>
+      <c r="D173" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E173">
+        <v>335000</v>
+      </c>
+      <c r="F173" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174">
+        <v>1776581182502</v>
+      </c>
+      <c r="B174" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C174" t="str">
+        <v>Alexander</v>
+      </c>
+      <c r="D174" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E174">
+        <v>70000</v>
+      </c>
+      <c r="F174" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175">
+        <v>1776581229719</v>
+      </c>
+      <c r="B175" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C175" t="str">
+        <v>Juanita</v>
+      </c>
+      <c r="D175" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E175">
+        <v>70000</v>
+      </c>
+      <c r="F175" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176">
+        <v>1776581283873</v>
+      </c>
+      <c r="B176" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C176" t="str">
+        <v>Jhojan</v>
+      </c>
+      <c r="D176" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E176">
+        <v>70000</v>
+      </c>
+      <c r="F176" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177">
+        <v>1776581318485</v>
+      </c>
+      <c r="B177" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C177" t="str">
+        <v>Fredy</v>
+      </c>
+      <c r="D177" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E177">
+        <v>70000</v>
+      </c>
+      <c r="F177" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178">
+        <v>1776581351190</v>
+      </c>
+      <c r="B178" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C178" t="str">
+        <v>Valeria</v>
+      </c>
+      <c r="D178" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E178">
+        <v>70000</v>
+      </c>
+      <c r="F178" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179">
+        <v>1776581650756</v>
+      </c>
+      <c r="B179" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C179" t="str">
+        <v>Martha2</v>
+      </c>
+      <c r="D179" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E179">
+        <v>70000</v>
+      </c>
+      <c r="F179" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180">
+        <v>1776581673204</v>
+      </c>
+      <c r="B180" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C180" t="str">
+        <v>Luisa</v>
+      </c>
+      <c r="D180" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E180">
+        <v>80000</v>
+      </c>
+      <c r="F180" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181">
+        <v>1776581710850</v>
+      </c>
+      <c r="B181" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C181" t="str">
+        <v>Martha1</v>
+      </c>
+      <c r="D181" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E181">
+        <v>90000</v>
+      </c>
+      <c r="F181" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182">
+        <v>1776581728315</v>
+      </c>
+      <c r="B182" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C182" t="str">
+        <v>Juan</v>
+      </c>
+      <c r="D182" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E182">
+        <v>80000</v>
+      </c>
+      <c r="F182" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183">
+        <v>1776581746615</v>
+      </c>
+      <c r="B183" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C183" t="str">
+        <v>Dreisy</v>
+      </c>
+      <c r="D183" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E183">
+        <v>80000</v>
+      </c>
+      <c r="F183" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184">
+        <v>1776581784531</v>
+      </c>
+      <c r="B184" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C184" t="str">
+        <v>Julian</v>
+      </c>
+      <c r="D184" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E184">
+        <v>80000</v>
+      </c>
+      <c r="F184" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185">
+        <v>1776581813254</v>
+      </c>
+      <c r="B185" t="str">
+        <v>2026-04-19</v>
+      </c>
+      <c r="C185" t="str">
+        <v>Sebastian</v>
+      </c>
+      <c r="D185" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E185">
+        <v>150000</v>
+      </c>
+      <c r="F185" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F127"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F185"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizar dashboard, gastos e inventario: ajustes en HTML
</commit_message>
<xml_diff>
--- a/data/gastos.xlsx
+++ b/data/gastos.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F194"/>
+  <dimension ref="A1:F210"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4279,9 +4279,329 @@
         <v>Luisa-Dreisy</v>
       </c>
     </row>
+    <row r="195">
+      <c r="A195">
+        <v>1777163340717</v>
+      </c>
+      <c r="B195" t="str">
+        <v>2026-04-26</v>
+      </c>
+      <c r="C195" t="str">
+        <v>Zumo limon</v>
+      </c>
+      <c r="D195" t="str">
+        <v>Insumos</v>
+      </c>
+      <c r="E195">
+        <v>48000</v>
+      </c>
+      <c r="F195" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196">
+        <v>1777171930685</v>
+      </c>
+      <c r="B196" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C196" t="str">
+        <v>Vasos, Copas</v>
+      </c>
+      <c r="D196" t="str">
+        <v>Insumos</v>
+      </c>
+      <c r="E196">
+        <v>59000</v>
+      </c>
+      <c r="F196" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197">
+        <v>1777184180693</v>
+      </c>
+      <c r="B197" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C197" t="str">
+        <v>Julian</v>
+      </c>
+      <c r="D197" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E197">
+        <v>90000</v>
+      </c>
+      <c r="F197" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198">
+        <v>1777184193737</v>
+      </c>
+      <c r="B198" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C198" t="str">
+        <v>Martha</v>
+      </c>
+      <c r="D198" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E198">
+        <v>80000</v>
+      </c>
+      <c r="F198" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199">
+        <v>1777184204445</v>
+      </c>
+      <c r="B199" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C199" t="str">
+        <v>Valeria</v>
+      </c>
+      <c r="D199" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E199">
+        <v>70000</v>
+      </c>
+      <c r="F199" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200">
+        <v>1777184217853</v>
+      </c>
+      <c r="B200" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C200" t="str">
+        <v>Juanita</v>
+      </c>
+      <c r="D200" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E200">
+        <v>70000</v>
+      </c>
+      <c r="F200" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201">
+        <v>1777184229174</v>
+      </c>
+      <c r="B201" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C201" t="str">
+        <v>Alexander</v>
+      </c>
+      <c r="D201" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E201">
+        <v>70000</v>
+      </c>
+      <c r="F201" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202">
+        <v>1777184241026</v>
+      </c>
+      <c r="B202" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C202" t="str">
+        <v>Jhojan</v>
+      </c>
+      <c r="D202" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E202">
+        <v>70000</v>
+      </c>
+      <c r="F202" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203">
+        <v>1777184249968</v>
+      </c>
+      <c r="B203" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C203" t="str">
+        <v>Fredy</v>
+      </c>
+      <c r="D203" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E203">
+        <v>70000</v>
+      </c>
+      <c r="F203" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204">
+        <v>1777184262033</v>
+      </c>
+      <c r="B204" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C204" t="str">
+        <v>Stiven</v>
+      </c>
+      <c r="D204" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E204">
+        <v>70000</v>
+      </c>
+      <c r="F204" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205">
+        <v>1777184334572</v>
+      </c>
+      <c r="B205" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C205" t="str">
+        <v>Sebastian</v>
+      </c>
+      <c r="D205" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E205">
+        <v>150000</v>
+      </c>
+      <c r="F205" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206">
+        <v>1777184349448</v>
+      </c>
+      <c r="B206" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C206" t="str">
+        <v>Dreisy</v>
+      </c>
+      <c r="D206" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E206">
+        <v>80000</v>
+      </c>
+      <c r="F206" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207">
+        <v>1777184370299</v>
+      </c>
+      <c r="B207" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C207" t="str">
+        <v>Juan Carlos</v>
+      </c>
+      <c r="D207" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E207">
+        <v>80000</v>
+      </c>
+      <c r="F207" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208">
+        <v>1777184388383</v>
+      </c>
+      <c r="B208" t="str">
+        <v>2026-04-25</v>
+      </c>
+      <c r="C208" t="str">
+        <v>Luisa Maria</v>
+      </c>
+      <c r="D208" t="str">
+        <v>Nomina</v>
+      </c>
+      <c r="E208">
+        <v>80000</v>
+      </c>
+      <c r="F208" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209">
+        <v>1777234509060</v>
+      </c>
+      <c r="B209" t="str">
+        <v>2026-04-26</v>
+      </c>
+      <c r="C209" t="str">
+        <v>Arriendo</v>
+      </c>
+      <c r="D209" t="str">
+        <v>Arriendo</v>
+      </c>
+      <c r="E209">
+        <v>6700000</v>
+      </c>
+      <c r="F209" t="str">
+        <v>Jorge</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210">
+        <v>1777342327513</v>
+      </c>
+      <c r="B210" t="str">
+        <v>2026-04-27</v>
+      </c>
+      <c r="C210" t="str">
+        <v>Vasos, mezcladores, café, aromaticas</v>
+      </c>
+      <c r="D210" t="str">
+        <v>Cafeteria</v>
+      </c>
+      <c r="E210">
+        <v>114000</v>
+      </c>
+      <c r="F210" t="str">
+        <v>MarthaC</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F194"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F210"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizar dashboard, ajuste modal de control de ventas
</commit_message>
<xml_diff>
--- a/data/gastos.xlsx
+++ b/data/gastos.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F210"/>
+  <dimension ref="A1:F217"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4599,9 +4599,149 @@
         <v>MarthaC</v>
       </c>
     </row>
+    <row r="211">
+      <c r="A211">
+        <v>1777520365898</v>
+      </c>
+      <c r="B211" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="C211" t="str">
+        <v>Insumos (Empanadas)</v>
+      </c>
+      <c r="D211" t="str">
+        <v>Cafeteria</v>
+      </c>
+      <c r="E211">
+        <v>25000</v>
+      </c>
+      <c r="F211" t="str">
+        <v>MarthaC</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212">
+        <v>1777679490990</v>
+      </c>
+      <c r="B212" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="C212" t="str">
+        <v>Venta cafeteria</v>
+      </c>
+      <c r="D212" t="str">
+        <v>Cafeteria</v>
+      </c>
+      <c r="E212">
+        <v>312000</v>
+      </c>
+      <c r="F212" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213">
+        <v>1777679536207</v>
+      </c>
+      <c r="B213" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="C213" t="str">
+        <v>Zumo de limon</v>
+      </c>
+      <c r="D213" t="str">
+        <v>Insumos</v>
+      </c>
+      <c r="E213">
+        <v>30000</v>
+      </c>
+      <c r="F213" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214">
+        <v>1777679608565</v>
+      </c>
+      <c r="B214" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="C214" t="str">
+        <v>Barra</v>
+      </c>
+      <c r="D214" t="str">
+        <v>Otros</v>
+      </c>
+      <c r="E214">
+        <v>229000</v>
+      </c>
+      <c r="F214" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215">
+        <v>1777680464193</v>
+      </c>
+      <c r="B215" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="C215" t="str">
+        <v>Cafeteria</v>
+      </c>
+      <c r="D215" t="str">
+        <v>Cafeteria</v>
+      </c>
+      <c r="E215">
+        <v>17940</v>
+      </c>
+      <c r="F215" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216">
+        <v>1777680498679</v>
+      </c>
+      <c r="B216" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="C216" t="str">
+        <v>Cafeteria- huevos</v>
+      </c>
+      <c r="D216" t="str">
+        <v>Cafeteria</v>
+      </c>
+      <c r="E216">
+        <v>50000</v>
+      </c>
+      <c r="F216" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217">
+        <v>1777680544058</v>
+      </c>
+      <c r="B217" t="str">
+        <v>2026-04-29</v>
+      </c>
+      <c r="C217" t="str">
+        <v>Linterna</v>
+      </c>
+      <c r="D217" t="str">
+        <v>Insumos</v>
+      </c>
+      <c r="E217">
+        <v>15899</v>
+      </c>
+      <c r="F217" t="str">
+        <v>Luisa-Dreisy</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F210"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F217"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>